<commit_message>
Add login smoke test
</commit_message>
<xml_diff>
--- a/src/test/java/test-cases/Login-Test-Cases.xlsx
+++ b/src/test/java/test-cases/Login-Test-Cases.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18168" windowHeight="2664"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Test Case</t>
   </si>
@@ -82,13 +83,27 @@
   </si>
   <si>
     <t>Valid email / Valid password</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_001
+      ↓
+HomePage
+      ↓
+Login sayfasına git
+      ↓
+Geçerli email + password
+      ↓
+Login
+      ↓
+"My Account" görünür mü?
+      ↓</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,13 +111,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -117,8 +146,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,7 +467,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -444,9 +477,13 @@
       <c r="C2" t="s">
         <v>19</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="E2" t="s">
         <v>20</v>
       </c>
+      <c r="F2" s="2"/>
       <c r="G2" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Add negative login test cases
</commit_message>
<xml_diff>
--- a/src/test/java/test-cases/Login-Test-Cases.xlsx
+++ b/src/test/java/test-cases/Login-Test-Cases.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18168" windowHeight="2664"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22464" windowHeight="7872"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>Test Case</t>
   </si>
@@ -98,12 +98,52 @@
 "My Account" görünür mü?
       ↓</t>
   </si>
+  <si>
+    <t>1. Login sayfasına git
+2. Geçerli email gir
+3. Geçersiz şifre gir
+4. Login butonuna tıkla</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Deneme1@gmail.com
+Password: Deneme</t>
+  </si>
+  <si>
+    <t>1. Login sayfasına git
+2. Geçersiz email gir
+3. Şifre gir
+4. Login butonuna tıkla</t>
+  </si>
+  <si>
+    <t>yanlis@gmail.com
+Password: Deneme1</t>
+  </si>
+  <si>
+    <t>1. Login sayfasına git
+2. Email alanını boş bırak
+3. Şifre gir
+4. Login butonuna tıkla</t>
+  </si>
+  <si>
+    <t>1. Login sayfasına git
+2. Email gir
+3. Password alanını boş bırak
+4. Login butonuna tıkla</t>
+  </si>
+  <si>
+    <t>Email: boş
+Password: Deneme1</t>
+  </si>
+  <si>
+    <t>Deneme1@gmail.com
+Password: boş</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,6 +157,26 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -143,17 +203,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -433,7 +501,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.109375" bestFit="1" customWidth="1"/>
@@ -444,7 +512,7 @@
     <col min="7" max="7" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -467,7 +535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="302.39999999999998">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -488,52 +556,96 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="158.4">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="2"/>
       <c r="G3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="144">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2"/>
       <c r="G4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="144">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2"/>
       <c r="G5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="172.8">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>15</v>
       </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="2"/>
       <c r="G6" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E4" r:id="rId1"/>
+    <hyperlink ref="E6" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>